<commit_message>
Fix Log4j dependency vulnerability
</commit_message>
<xml_diff>
--- a/SwagLabsProject/src/test/resources/TestData_AllModules.xlsx
+++ b/SwagLabsProject/src/test/resources/TestData_AllModules.xlsx
@@ -1,21 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\SwagLabs_IntelliJ_Fixed\SwagLabsProject\SwagLabsProject\src\test\resources\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51526CA8-7DBF-4F1F-9370-F9BBCBF711F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="LoginData" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="ProductData" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="CartData" sheetId="3" r:id="rId6"/>
-    <sheet state="visible" name="CheckoutData" sheetId="4" r:id="rId7"/>
-    <sheet state="visible" name="HamburgerData" sheetId="5" r:id="rId8"/>
+    <sheet name="LoginData" sheetId="1" r:id="rId1"/>
+    <sheet name="ProductData" sheetId="2" r:id="rId2"/>
+    <sheet name="CartData" sheetId="3" r:id="rId3"/>
+    <sheet name="CheckoutData" sheetId="4" r:id="rId4"/>
+    <sheet name="HamburgerData" sheetId="5" r:id="rId5"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="87">
   <si>
     <t>TestCase</t>
   </si>
@@ -164,15 +173,6 @@
     <t>TC-CHK-02</t>
   </si>
   <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>Doe</t>
-  </si>
-  <si>
-    <t>560001</t>
-  </si>
-  <si>
     <t>TC-CHK-03</t>
   </si>
   <si>
@@ -237,21 +237,70 @@
   </si>
   <si>
     <t>TC-HAM-11</t>
+  </si>
+  <si>
+    <t>Vishwa</t>
+  </si>
+  <si>
+    <t>Bohaddur</t>
+  </si>
+  <si>
+    <t>srinivas</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>Raj</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>kiran</t>
+  </si>
+  <si>
+    <t>raj</t>
+  </si>
+  <si>
+    <t>Virat</t>
+  </si>
+  <si>
+    <t>Kohli</t>
+  </si>
+  <si>
+    <t>ram</t>
+  </si>
+  <si>
+    <t>Charan</t>
+  </si>
+  <si>
+    <t>raja</t>
+  </si>
+  <si>
+    <t>Arjun</t>
+  </si>
+  <si>
+    <t>Ashoke</t>
+  </si>
+  <si>
+    <t>Sharma</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2">
     <font>
-      <sz val="11.0"/>
-      <color/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -259,59 +308,52 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -467,7 +509,7 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln cap="flat" cmpd="sng" w="9525" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -476,13 +518,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln cap="flat" cmpd="sng" w="25400" algn="ctr">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln cap="flat" cmpd="sng" w="38100" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -492,7 +534,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" rotWithShape="0" dir="5400000" dist="20000">
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -501,7 +543,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" rotWithShape="0" dir="5400000" dist="23000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -510,7 +552,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" rotWithShape="0" dir="5400000" dist="23000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -520,12 +562,12 @@
             <a:camera prst="orthographicFront">
               <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
+            <a:lightRig rig="threePt" dir="t">
               <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
-            <a:bevelT h="25400" w="63500"/>
+            <a:bevelT w="63500" h="25400"/>
           </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
@@ -556,7 +598,7 @@
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
-            <a:fillToRect b="180000" l="50000" r="50000" t="-80000"/>
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
@@ -575,7 +617,7 @@
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
-            <a:fillToRect b="50000" l="50000" r="50000" t="50000"/>
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
@@ -587,19 +629,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C100"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="14.0"/>
-    <col customWidth="1" min="2" max="2" width="16.0"/>
-    <col customWidth="1" min="3" max="3" width="17.0"/>
-    <col customWidth="1" min="4" max="11" width="8.71"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="11" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" ht="14.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -610,12 +650,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" ht="14.5">
       <c r="A2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3" ht="14.5">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -626,7 +666,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:3" ht="14.5">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -637,7 +677,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:3" ht="14.5">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -648,7 +688,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:3" ht="14.5">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -659,7 +699,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:3" ht="14.5">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -667,7 +707,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:3" ht="14.5">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -675,7 +715,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:3" ht="14.5">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -686,7 +726,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:3" ht="14.5">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -697,7 +737,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:3" ht="14.5">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -783,27 +823,23 @@
     <row r="99" ht="15.75" customHeight="1"/>
     <row r="100" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:C100"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="13.0"/>
-    <col customWidth="1" min="2" max="2" width="22.0"/>
-    <col customWidth="1" min="3" max="3" width="14.0"/>
-    <col customWidth="1" min="4" max="11" width="8.71"/>
+    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="11" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" ht="14.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -814,12 +850,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" ht="14.5">
       <c r="A2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3" ht="14.5">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -827,7 +863,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:3" ht="14.5">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -835,7 +871,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:3" ht="14.5">
       <c r="A5" t="s">
         <v>23</v>
       </c>
@@ -843,7 +879,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:3" ht="14.5">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -851,7 +887,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:3" ht="14.5">
       <c r="A7" t="s">
         <v>26</v>
       </c>
@@ -859,7 +895,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:3" ht="14.5">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -867,7 +903,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:3" ht="14.5">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -875,7 +911,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:3" ht="14.5">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -883,7 +919,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:3" ht="14.5">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -972,26 +1008,22 @@
     <row r="99" ht="15.75" customHeight="1"/>
     <row r="100" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:B100"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="13.0"/>
-    <col customWidth="1" min="2" max="2" width="22.0"/>
-    <col customWidth="1" min="3" max="11" width="8.71"/>
+    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="11" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" ht="14.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -999,7 +1031,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" ht="14.5">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -1007,7 +1039,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" ht="14.5">
       <c r="A3" t="s">
         <v>35</v>
       </c>
@@ -1015,7 +1047,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" ht="14.5">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -1023,12 +1055,12 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:2" ht="14.5">
       <c r="A5" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:2" ht="14.5">
       <c r="A6" t="s">
         <v>38</v>
       </c>
@@ -1036,7 +1068,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:2" ht="14.5">
       <c r="A7" t="s">
         <v>39</v>
       </c>
@@ -1044,7 +1076,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:2" ht="14.5">
       <c r="A8" t="s">
         <v>40</v>
       </c>
@@ -1052,7 +1084,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:2" ht="14.5">
       <c r="A9" t="s">
         <v>41</v>
       </c>
@@ -1060,7 +1092,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:2" ht="14.5">
       <c r="A10" t="s">
         <v>42</v>
       </c>
@@ -1068,7 +1100,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:2" ht="14.5">
       <c r="A11" t="s">
         <v>43</v>
       </c>
@@ -1157,27 +1189,23 @@
     <row r="99" ht="15.75" customHeight="1"/>
     <row r="100" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:D100"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="2" width="12.0"/>
-    <col customWidth="1" min="3" max="3" width="11.0"/>
-    <col customWidth="1" min="4" max="4" width="10.0"/>
-    <col customWidth="1" min="5" max="11" width="8.71"/>
+    <col min="1" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="11" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:4" ht="14.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1191,159 +1219,159 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:4" ht="14.5">
       <c r="A2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:4" ht="14.5">
       <c r="A3" t="s">
         <v>48</v>
       </c>
       <c r="B3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3">
+        <v>234455</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="14.5">
+      <c r="A4" t="s">
         <v>49</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D4">
+        <v>543433</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="14.5">
+      <c r="A5" t="s">
         <v>50</v>
       </c>
-      <c r="D3" t="s">
+      <c r="B5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D5">
+        <v>343431</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="14.5">
+      <c r="A6" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
+      <c r="B6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D6">
+        <v>911231</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="14.5">
+      <c r="A7" t="s">
         <v>52</v>
       </c>
-      <c r="B4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
+      <c r="B7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7">
+        <v>545221</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="14.5">
+      <c r="A8" t="s">
         <v>53</v>
       </c>
-      <c r="B5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
+      <c r="B8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D8">
+        <v>456001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="14.5">
+      <c r="A9" t="s">
         <v>54</v>
       </c>
-      <c r="B6" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" t="s">
-        <v>50</v>
-      </c>
-      <c r="D6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
+      <c r="C9" t="s">
+        <v>83</v>
+      </c>
+      <c r="D9">
+        <v>676877</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="14.5">
+      <c r="A10" t="s">
         <v>55</v>
       </c>
-      <c r="B7" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
+      <c r="B10" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10">
+        <v>364251</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="14.5">
+      <c r="A11" t="s">
         <v>56</v>
       </c>
-      <c r="B8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
+      <c r="B11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="14.5">
+      <c r="A12" t="s">
         <v>57</v>
       </c>
-      <c r="C9" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
+      <c r="B12" t="s">
+        <v>84</v>
+      </c>
+      <c r="C12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12">
+        <v>456321</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="14.5">
+      <c r="A13" t="s">
         <v>58</v>
       </c>
-      <c r="B10" t="s">
-        <v>49</v>
-      </c>
-      <c r="D10" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
+      <c r="B13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D13">
+        <v>788233</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="14.5">
+      <c r="A14" t="s">
         <v>59</v>
-      </c>
-      <c r="B11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C11" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>60</v>
-      </c>
-      <c r="B12" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12" t="s">
-        <v>50</v>
-      </c>
-      <c r="D12" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>61</v>
-      </c>
-      <c r="B13" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13" t="s">
-        <v>50</v>
-      </c>
-      <c r="D13" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1427,26 +1455,22 @@
     <row r="99" ht="15.75" customHeight="1"/>
     <row r="100" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:B100"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="12.0"/>
-    <col customWidth="1" min="2" max="2" width="22.0"/>
-    <col customWidth="1" min="3" max="11" width="8.71"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="11" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" ht="14.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1454,71 +1478,71 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" ht="14.5">
       <c r="A2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="14.5">
+      <c r="A3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="14.5">
+      <c r="A4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="14.5">
+      <c r="A5" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="s">
+    <row r="6" spans="1:2" ht="14.5">
+      <c r="A6" t="s">
         <v>64</v>
       </c>
-      <c r="B3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
+    </row>
+    <row r="7" spans="1:2" ht="14.5">
+      <c r="A7" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="s">
+    <row r="8" spans="1:2" ht="14.5">
+      <c r="A8" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="14.5">
+      <c r="A9" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="s">
+    <row r="10" spans="1:2" ht="14.5">
+      <c r="A10" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="14.5">
+      <c r="A11" t="s">
         <v>69</v>
       </c>
-      <c r="B8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="14.5">
+      <c r="A12" t="s">
         <v>70</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>71</v>
-      </c>
-      <c r="B10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>72</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>73</v>
       </c>
       <c r="B12" t="s">
         <v>21</v>
@@ -1605,9 +1629,7 @@
     <row r="99" ht="15.75" customHeight="1"/>
     <row r="100" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>